<commit_message>
Deploy browser work-order matching website
</commit_message>
<xml_diff>
--- a/downloads/AutoReport_sample_results.xlsx
+++ b/downloads/AutoReport_sample_results.xlsx
@@ -487,32 +487,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -532,32 +524,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Slate/Congo 14</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[{"機種": "Slate/Congo 14", "IC": "Goodix", "產品系列": ["CY26"], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 2, "原始IC／機型": "CY26Goodix", "整理依據": ["IC／機型原文含代別；已分離代別與 IC 品牌"]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C514-260400001", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C514-260400001", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 2}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -577,32 +561,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Jarvis 16</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[{"機種": "Jarvis 16", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C533-250800002", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C533-250800002", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 4}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -622,32 +598,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Synaptics</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 3, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C533-251200001", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C533-251200001", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 3}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -667,32 +635,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Echo wired mouse</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Elan</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[{"機種": "Echo wired mouse", "IC": "Elan", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 3, "原始IC／機型": "Elan", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C515-251100001", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C515-251100001", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 3}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -712,32 +672,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Synaptics</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 136, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C516-626070202", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C516-626070202", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 136}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -757,32 +709,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>CY26-14</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Synaptics</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[{"機種": "CY26-14", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 40, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "626090006", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "626090006", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 40}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -802,32 +746,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>CY26</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[{"機種": "CY26", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 50, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [138, 141, 174, 175, 193, 197, 209, 219, 239, 360, 367]}]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C630-626080041", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C630-626080041", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 50}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -847,32 +783,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 5, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 8, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 10, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 11, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 12, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 13, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 14, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 17, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 18, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 19, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 20, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 21, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 22, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 23, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 27, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 43, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 48, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 53, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 61, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 62, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 63, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 64, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 65, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 66, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 68, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 76, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 77, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 89, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 90, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 93, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 94, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 96, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 105, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 106, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 108, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 112, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 116, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 120, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 124, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 125, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 128, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 129, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 137, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 140, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 6, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 7, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 10, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 15, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 26, "原始IC／機型": "", "整理依據": ["以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [1, 2, 5, 7, 8, 9, 10, 11, 14, 15, 16, 17, 18, 19, 20, 24, 40, 45, 50, 58, 59, 60, 61, 62, 63, 65, 73, 74, 86, 87, 90, 91, 93, 102, 103, 105, 109, 113, 117, 121, 122, 125, 126, 134, 137, 283, 285, 286, 289, 294]}]}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 30, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [1, 2, 5, 7, 8, 9, 10, 11, 14, 15, 16, 17, 18, 19, 20, 24, 40, 45, 50, 58, 59, 60, 61, 62, 63, 65, 73, 74, 86, 87, 90, 91, 93, 102, 103, 105, 109, 113, 117, 121, 122, 125, 126, 134, 137, 283, 285, 286, 289, 294]}]}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 43, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [1, 2, 5, 7, 8, 9, 10, 11, 14, 15, 16, 17, 18, 19, 20, 24, 40, 45, 50, 58, 59, 60, 61, 62, 63, 65, 73, 74, 86, 87, 90, 91, 93, 102, 103, 105, 109, 113, 117, 121, 122, 125, 126, 134, 137, 283, 285, 286, 289, 294]}]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "part", "查找值": "98000320-107", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "part", "查找值": "98000320-107", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 5}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 10}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 11}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 12}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 13}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 14}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 17}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 18}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 19}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 20}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 21}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 23}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 27}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 43}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 48}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 53}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 61}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 62}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 63}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 64}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 65}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 66}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 68}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 76}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 77}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 89}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 90}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 93}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 94}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 96}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 105}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 106}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 108}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 112}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 116}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 120}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 124}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 125}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 128}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 129}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 137}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 140}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 4}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 6}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 7}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 10}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 15}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 26}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 43}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -892,24 +820,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>多組候選</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 13", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 9, "原始IC／機型": "Goodix", "整理依據": []}]}, {"機種": "Taroko 13", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 8, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C533-260100003", "找到候選組數": 2}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C533-260100003", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 9}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -929,24 +857,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>來源未提供完整對應</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[{"機種": "CY26", "IC": "", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 52, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "IC 待確認：料號對應多個 IC"]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C630-626080043", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C630-626080043", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 52}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -966,24 +894,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>來源未提供完整對應</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[{"機種": "", "IC": "Elan", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 30, "原始IC／機型": "Elan", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 31, "原始IC／機型": "Elan", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C510-260500009", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C510-260500009", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 31}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1040,7 +968,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>條件不一致</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1052,12 +980,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 1}, {"欄位類別": "ic", "查找值": "Synaptics", "找到候選組數": 11}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 0}, {"欄位類別": "ic", "查找值": "Synaptics", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 9}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 16}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 29}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 32}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 33}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 36}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 37}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 38}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 50}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 67}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 71}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 72}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 73}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 78}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 82}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 83}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 84}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 85}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 86}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 92}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 95}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 97}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 99}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 102}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 103}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 107}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 114}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 119}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 121}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 122}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 123}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 130}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 131}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 132}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 133}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 136}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 139}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 9}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 10}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 11}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 16}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 17}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 18}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 19}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 23}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 31}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 32}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 40}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 41}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 42}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 43}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 49}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 50}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 51}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 53}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 58}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 59}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 62}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 64}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 65}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 66}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 67}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 70}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 78}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 80}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 81}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 82}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 84}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 87}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 88}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 92}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 97}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 98}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 99}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 101}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 3}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 12}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 13}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 17}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 21}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 24}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 32}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 33}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 34}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 37}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 42}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 46}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 47}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 53}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 57}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 7}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 12}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 14}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 19}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 20}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 21}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 23}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 24}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 29}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 31}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 34}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 37}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 38}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 40}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 41}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 45}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 49}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 51}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">

</xml_diff>

<commit_message>
Reset reference database and clear legacy browser data once
</commit_message>
<xml_diff>
--- a/downloads/AutoReport_sample_results.xlsx
+++ b/downloads/AutoReport_sample_results.xlsx
@@ -487,32 +487,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -532,32 +524,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Slate/Congo 14</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[{"機種": "Slate/Congo 14", "IC": "Goodix", "產品系列": ["CY26"], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 2, "原始IC／機型": "CY26Goodix", "整理依據": ["IC／機型原文含代別；已分離代別與 IC 品牌"]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C514-260400001", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C514-260400001", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 2}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -577,32 +561,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Jarvis 16</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[{"機種": "Jarvis 16", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C533-250800002", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C533-250800002", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 4}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -622,32 +598,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Synaptics</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 3, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C533-251200001", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C533-251200001", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 3}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -667,32 +635,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Echo wired mouse</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Elan</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[{"機種": "Echo wired mouse", "IC": "Elan", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 3, "原始IC／機型": "Elan", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C515-251100001", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C515-251100001", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 3}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -712,32 +672,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Synaptics</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 136, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C516-626070202", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C516-626070202", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 136}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -757,32 +709,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>CY26-14</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Synaptics</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[{"機種": "CY26-14", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 40, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "626090006", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "626090006", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 40}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -802,32 +746,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>CY26</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[{"機種": "CY26", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 50, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [138, 141, 174, 175, 193, 197, 209, 219, 239, 360, 367]}]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C630-626080041", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C630-626080041", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 50}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -847,32 +783,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>唯一匹配</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Taroko 14</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Goodix</t>
-        </is>
-      </c>
+          <t>查無資料</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 14", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 5, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 8, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 10, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 11, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 12, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 13, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 14, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 17, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 18, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 19, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 20, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 21, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 22, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 23, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 27, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 43, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 48, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 53, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 61, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 62, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 63, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 64, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 65, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 66, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 68, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 76, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 77, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 89, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 90, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 93, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 94, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 96, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 105, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 106, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 108, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 112, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 116, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 120, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 124, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 125, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 128, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 129, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 137, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 140, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 4, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 6, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 7, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 10, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 15, "原始IC／機型": "Goodix", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 26, "原始IC／機型": "", "整理依據": ["以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [1, 2, 5, 7, 8, 9, 10, 11, 14, 15, 16, 17, 18, 19, 20, 24, 40, 45, 50, 58, 59, 60, 61, 62, 63, 65, 73, 74, 86, 87, 90, 91, 93, 102, 103, 105, 109, 113, 117, 121, 122, 125, 126, 134, 137, 283, 285, 286, 289, 294]}]}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 30, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [1, 2, 5, 7, 8, 9, 10, 11, 14, 15, 16, 17, 18, 19, 20, 24, 40, 45, 50, 58, 59, 60, 61, 62, 63, 65, 73, 74, 86, 87, 90, 91, 93, 102, 103, 105, 109, 113, 117, 121, 122, 125, 126, 134, 137, 283, 285, 286, 289, 294]}]}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 43, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "以相同主料號／DPN 跨頁確認 IC：Goodix", {"IC依據資料列ID": [1, 2, 5, 7, 8, 9, 10, 11, 14, 15, 16, 17, 18, 19, 20, 24, 40, 45, 50, 58, 59, 60, 61, 62, 63, 65, 73, 74, 86, 87, 90, 91, 93, 102, 103, 105, 109, 113, 117, 121, 122, 125, 126, 134, 137, 283, 285, 286, 289, 294]}]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "part", "查找值": "98000320-107", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "part", "查找值": "98000320-107", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 5}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 10}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 11}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 12}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 13}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 14}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 17}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 18}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 19}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 20}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 21}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 23}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 27}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 43}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 48}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 53}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 61}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 62}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 63}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 64}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 65}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 66}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 68}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 76}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 77}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 89}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 90}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 93}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 94}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 96}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 105}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 106}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 108}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 112}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 116}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 120}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 124}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 125}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 128}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 129}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 137}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 140}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 4}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 6}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 7}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 10}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 15}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 26}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 43}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -892,24 +820,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>多組候選</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[{"機種": "Taroko 13", "IC": "Goodix", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 9, "原始IC／機型": "Goodix", "整理依據": []}]}, {"機種": "Taroko 13", "IC": "Synaptics", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 8, "原始IC／機型": "Synaptics", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C533-260100003", "找到候選組數": 2}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C533-260100003", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 9}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -929,24 +857,24 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>來源未提供完整對應</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[{"機種": "CY26", "IC": "", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 52, "原始IC／機型": "不良品返修", "整理依據": ["原始 IC 欄為重工用途，需依料號確認", "IC 待確認：料號對應多個 IC"]}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C630-626080043", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C630-626080043", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 52}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -966,24 +894,24 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>來源未提供完整對應</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[{"機種": "", "IC": "Elan", "產品系列": [], "來源": [{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 30, "原始IC／機型": "Elan", "整理依據": []}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 31, "原始IC／機型": "Elan", "整理依據": []}]}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C510-260500009", "找到候選組數": 1}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C510-260500009", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（CY24&amp;25）", "列號": 31}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1040,7 +968,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>條件不一致</t>
+          <t>查無資料</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1052,12 +980,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 1}, {"欄位類別": "ic", "查找值": "Synaptics", "找到候選組數": 11}]</t>
+          <t>[{"欄位類別": "order", "查找值": "C515-250300004", "找到候選組數": 0}, {"欄位類別": "ic", "查找值": "Synaptics", "找到候選組數": 0}]</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[{"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 4}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 9}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 16}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 29}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 32}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 33}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 36}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 37}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 38}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 50}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 67}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 71}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 72}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 73}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 78}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 82}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 83}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 84}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 85}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 86}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 92}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 95}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 97}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 99}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 102}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 103}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 107}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 114}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 119}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 121}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 122}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 123}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 130}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 131}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 132}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 133}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 136}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "工单（A16）", "列號": 139}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 9}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 10}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 11}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 16}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 17}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 18}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 19}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 23}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 31}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 32}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 40}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 41}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 42}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 43}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 49}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 50}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 51}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 53}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 58}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 59}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 62}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 64}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 65}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 66}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 67}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 70}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 78}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 80}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 81}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 82}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 84}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 87}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 88}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 92}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 97}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 98}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 99}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "CY26", "列號": 101}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 3}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 8}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 12}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 13}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 17}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 21}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 24}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 32}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 33}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 34}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 37}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 42}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 46}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 47}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 53}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "重工工单1", "列號": 57}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 7}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 12}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 14}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 19}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 20}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 21}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 22}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 23}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 24}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 29}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 30}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 31}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 34}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 37}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 38}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 40}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 41}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 45}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 49}, {"檔案": "工單明细表_中科廠-2026.xlsx", "分頁": "NPI", "列號": 51}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">

</xml_diff>